<commit_message>
feat: harden JWT security with rate limiting and token blacklist
- Add login/register rate throttling (5/min and 3/hour)
- Shorten access token lifetime from 1 day to 30 minutes
- Enable token blacklist to invalidate rotated refresh tokens
- Update PI template file

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/sea_saw_export/templates/PI_template.xlsx
+++ b/app/sea_saw_export/templates/PI_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coolister/Desktop/sea-saw/sea-saw-server/app/sea_saw_sales/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coolister/Desktop/sea-saw/sea-saw-server/app/sea_saw_export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15E6538-DC3C-FD40-A959-B88F0FE6085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F560E81-C4FA-CD41-88B2-E2A78BA721CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2640" yWindow="-20060" windowWidth="31740" windowHeight="18480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1840" yWindow="880" windowWidth="21300" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEMPLATE" sheetId="3" r:id="rId1"/>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
-    <t>Invoice No</t>
-  </si>
-  <si>
     <t>Issue Date</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>Room B, 15/F, Kin Hing Industrial Building, 17-23 Shek Kin Street, Kwai Chung, HongKong</t>
   </si>
   <si>
-    <t>PROFORMA INVOICE</t>
-  </si>
-  <si>
     <t>Seller</t>
   </si>
   <si>
@@ -128,6 +122,14 @@
   <si>
     <t xml:space="preserve">Dispute Resolution: Any disputes arising from this contract shall be resolved through friendly negotiation.
 </t>
+  </si>
+  <si>
+    <t>SALES CONTRACT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Contract No</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -969,21 +971,61 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="4" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="27" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="9" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="43" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="178" fontId="19" fillId="2" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="177" fontId="19" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="176" fontId="27" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1007,46 +1049,6 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="177" fontId="19" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="178" fontId="4" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="27" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="43" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="19" fillId="2" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1071,53 +1073,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>289983</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>124884</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1265768" cy="1272629"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="图片 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1915583" y="10310284"/>
-          <a:ext cx="1265768" cy="1272629"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1459,42 +1414,42 @@
     </row>
     <row r="2" spans="1:9" s="5" customFormat="1" ht="46" customHeight="1">
       <c r="A2" s="4"/>
-      <c r="B2" s="124" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="125"/>
+      <c r="B2" s="104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" ht="15" customHeight="1">
       <c r="A3" s="4"/>
-      <c r="B3" s="132" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="125"/>
-      <c r="D3" s="125"/>
-      <c r="E3" s="125"/>
-      <c r="F3" s="125"/>
-      <c r="G3" s="125"/>
-      <c r="H3" s="125"/>
-      <c r="I3" s="125"/>
+      <c r="B3" s="116" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="105"/>
+      <c r="D3" s="105"/>
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
     </row>
     <row r="4" spans="1:9" s="5" customFormat="1" ht="31" customHeight="1">
       <c r="A4" s="4"/>
-      <c r="B4" s="131" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="125"/>
-      <c r="D4" s="125"/>
-      <c r="E4" s="125"/>
-      <c r="F4" s="125"/>
-      <c r="G4" s="125"/>
-      <c r="H4" s="125"/>
-      <c r="I4" s="125"/>
+      <c r="B4" s="115" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="105"/>
+      <c r="D4" s="105"/>
+      <c r="E4" s="105"/>
+      <c r="F4" s="105"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="105"/>
+      <c r="I4" s="105"/>
     </row>
     <row r="5" spans="1:9" ht="10" customHeight="1">
       <c r="B5" s="6"/>
@@ -1509,7 +1464,7 @@
     <row r="6" spans="1:9" s="16" customFormat="1" ht="30" customHeight="1">
       <c r="A6" s="11"/>
       <c r="B6" s="67" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -1518,7 +1473,7 @@
       <c r="G6" s="73"/>
       <c r="H6" s="74"/>
       <c r="I6" s="75" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="16" customFormat="1" ht="20" customHeight="1">
@@ -1528,46 +1483,46 @@
       <c r="D7" s="63"/>
       <c r="E7" s="64"/>
       <c r="F7" s="76" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G7" s="77"/>
       <c r="H7" s="76" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="77"/>
     </row>
     <row r="8" spans="1:9" s="16" customFormat="1" ht="20" customHeight="1">
       <c r="A8" s="11"/>
-      <c r="B8" s="113"/>
-      <c r="C8" s="114"/>
-      <c r="D8" s="114"/>
-      <c r="E8" s="114"/>
-      <c r="F8" s="104"/>
-      <c r="G8" s="105"/>
+      <c r="B8" s="129"/>
+      <c r="C8" s="130"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="130"/>
+      <c r="F8" s="125"/>
+      <c r="G8" s="114"/>
       <c r="H8" s="79"/>
       <c r="I8" s="65"/>
     </row>
     <row r="9" spans="1:9" s="16" customFormat="1" ht="20" customHeight="1">
       <c r="A9" s="11"/>
-      <c r="B9" s="108"/>
-      <c r="C9" s="114"/>
-      <c r="D9" s="114"/>
-      <c r="E9" s="114"/>
+      <c r="B9" s="110"/>
+      <c r="C9" s="130"/>
+      <c r="D9" s="130"/>
+      <c r="E9" s="130"/>
       <c r="F9" s="76" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="80"/>
       <c r="H9" s="76" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="81"/>
     </row>
     <row r="10" spans="1:9" s="18" customFormat="1" ht="20" customHeight="1">
       <c r="A10" s="17"/>
-      <c r="B10" s="109"/>
-      <c r="C10" s="110"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="110"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="122"/>
+      <c r="D10" s="122"/>
+      <c r="E10" s="122"/>
       <c r="F10" s="78"/>
       <c r="G10" s="66"/>
       <c r="H10" s="32"/>
@@ -1587,13 +1542,13 @@
     <row r="12" spans="1:9" s="20" customFormat="1" ht="30" customHeight="1">
       <c r="A12" s="21"/>
       <c r="B12" s="67" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="67" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
@@ -1612,38 +1567,38 @@
     </row>
     <row r="14" spans="1:9" s="20" customFormat="1" ht="18" customHeight="1">
       <c r="A14" s="21"/>
-      <c r="B14" s="136"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="107"/>
-      <c r="E14" s="103"/>
-      <c r="F14" s="117"/>
-      <c r="G14" s="107"/>
-      <c r="H14" s="107"/>
-      <c r="I14" s="103"/>
+      <c r="B14" s="120"/>
+      <c r="C14" s="103"/>
+      <c r="D14" s="103"/>
+      <c r="E14" s="121"/>
+      <c r="F14" s="133"/>
+      <c r="G14" s="103"/>
+      <c r="H14" s="103"/>
+      <c r="I14" s="121"/>
     </row>
     <row r="15" spans="1:9" s="20" customFormat="1" ht="36" customHeight="1">
       <c r="A15" s="21"/>
-      <c r="B15" s="109"/>
-      <c r="C15" s="110"/>
-      <c r="D15" s="110"/>
-      <c r="E15" s="105"/>
-      <c r="F15" s="108"/>
-      <c r="G15" s="107"/>
-      <c r="H15" s="107"/>
-      <c r="I15" s="103"/>
+      <c r="B15" s="113"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="114"/>
+      <c r="F15" s="110"/>
+      <c r="G15" s="103"/>
+      <c r="H15" s="103"/>
+      <c r="I15" s="121"/>
     </row>
     <row r="16" spans="1:9" s="20" customFormat="1" ht="20" customHeight="1">
       <c r="A16" s="21"/>
       <c r="B16" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16" s="82"/>
       <c r="D16" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="83"/>
       <c r="F16" s="24" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G16" s="84"/>
       <c r="H16" s="85"/>
@@ -1663,11 +1618,11 @@
     <row r="18" spans="1:11" s="20" customFormat="1" ht="20" customHeight="1">
       <c r="A18" s="21"/>
       <c r="B18" s="24" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C18" s="82"/>
       <c r="D18" s="24" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E18" s="83"/>
       <c r="F18" s="93"/>
@@ -1688,46 +1643,46 @@
     </row>
     <row r="20" spans="1:11" s="26" customFormat="1" ht="20" customHeight="1">
       <c r="A20" s="25"/>
-      <c r="B20" s="128" t="s">
+      <c r="B20" s="108" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="109"/>
+      <c r="D20" s="111" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="112"/>
+      <c r="F20" s="106" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="107"/>
+      <c r="H20" s="127" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="129"/>
-      <c r="D20" s="130" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="122"/>
-      <c r="F20" s="126" t="s">
+      <c r="I20" s="127" t="s">
         <v>24</v>
-      </c>
-      <c r="G20" s="127"/>
-      <c r="H20" s="111" t="s">
-        <v>25</v>
-      </c>
-      <c r="I20" s="111" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="20" customFormat="1" ht="20" customHeight="1">
       <c r="A21" s="21"/>
-      <c r="B21" s="108"/>
-      <c r="C21" s="107"/>
-      <c r="D21" s="109"/>
-      <c r="E21" s="105"/>
+      <c r="B21" s="110"/>
+      <c r="C21" s="103"/>
+      <c r="D21" s="113"/>
+      <c r="E21" s="114"/>
       <c r="F21" s="36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G21" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="H21" s="112"/>
-      <c r="I21" s="112"/>
+        <v>25</v>
+      </c>
+      <c r="H21" s="128"/>
+      <c r="I21" s="128"/>
     </row>
     <row r="22" spans="1:11" s="20" customFormat="1" ht="84" customHeight="1">
       <c r="A22" s="21"/>
-      <c r="B22" s="133"/>
-      <c r="C22" s="134"/>
-      <c r="D22" s="135"/>
-      <c r="E22" s="134"/>
+      <c r="B22" s="117"/>
+      <c r="C22" s="118"/>
+      <c r="D22" s="119"/>
+      <c r="E22" s="118"/>
       <c r="F22" s="38"/>
       <c r="G22" s="39">
         <f>F22*20</f>
@@ -1741,10 +1696,10 @@
     </row>
     <row r="23" spans="1:11" s="20" customFormat="1" ht="25" customHeight="1">
       <c r="A23" s="21"/>
-      <c r="B23" s="115"/>
-      <c r="C23" s="116"/>
-      <c r="D23" s="116"/>
-      <c r="E23" s="116"/>
+      <c r="B23" s="131"/>
+      <c r="C23" s="132"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="132"/>
       <c r="F23" s="99"/>
       <c r="G23" s="99"/>
       <c r="H23" s="99"/>
@@ -1753,52 +1708,52 @@
     <row r="24" spans="1:11" s="20" customFormat="1" ht="35" customHeight="1">
       <c r="A24" s="21"/>
       <c r="B24" s="101" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="34"/>
       <c r="D24" s="34"/>
       <c r="E24" s="41"/>
-      <c r="F24" s="137" t="s">
-        <v>28</v>
-      </c>
-      <c r="G24" s="105"/>
-      <c r="H24" s="118">
+      <c r="F24" s="123" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="114"/>
+      <c r="H24" s="134">
         <f>SUM(I22:I23)</f>
         <v>0</v>
       </c>
-      <c r="I24" s="103"/>
-      <c r="J24" s="123"/>
-      <c r="K24" s="107"/>
+      <c r="I24" s="121"/>
+      <c r="J24" s="102"/>
+      <c r="K24" s="103"/>
     </row>
     <row r="25" spans="1:11" s="20" customFormat="1" ht="33" customHeight="1">
       <c r="A25" s="21"/>
-      <c r="B25" s="119" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="107"/>
-      <c r="D25" s="107"/>
-      <c r="E25" s="103"/>
-      <c r="F25" s="121" t="s">
+      <c r="B25" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="103"/>
+      <c r="D25" s="103"/>
+      <c r="E25" s="121"/>
+      <c r="F25" s="137" t="s">
+        <v>6</v>
+      </c>
+      <c r="G25" s="112"/>
+      <c r="H25" s="137" t="s">
         <v>7</v>
       </c>
-      <c r="G25" s="122"/>
-      <c r="H25" s="121" t="s">
-        <v>8</v>
-      </c>
-      <c r="I25" s="122"/>
+      <c r="I25" s="112"/>
     </row>
     <row r="26" spans="1:11" s="28" customFormat="1" ht="33" customHeight="1">
       <c r="A26" s="27"/>
-      <c r="B26" s="108"/>
-      <c r="C26" s="120"/>
-      <c r="D26" s="120"/>
-      <c r="E26" s="103"/>
-      <c r="F26" s="102"/>
-      <c r="G26" s="103"/>
-      <c r="H26" s="102" t="s">
-        <v>13</v>
-      </c>
-      <c r="I26" s="103"/>
+      <c r="B26" s="110"/>
+      <c r="C26" s="136"/>
+      <c r="D26" s="136"/>
+      <c r="E26" s="121"/>
+      <c r="F26" s="124"/>
+      <c r="G26" s="121"/>
+      <c r="H26" s="124" t="s">
+        <v>12</v>
+      </c>
+      <c r="I26" s="121"/>
     </row>
     <row r="27" spans="1:11" s="20" customFormat="1" ht="7" customHeight="1">
       <c r="A27" s="21"/>
@@ -1814,7 +1769,7 @@
     <row r="28" spans="1:11" s="20" customFormat="1" ht="27" customHeight="1">
       <c r="A28" s="21"/>
       <c r="B28" s="67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -1826,36 +1781,36 @@
     </row>
     <row r="29" spans="1:11" s="20" customFormat="1" ht="25" customHeight="1">
       <c r="A29" s="21"/>
-      <c r="B29" s="106"/>
-      <c r="C29" s="107"/>
-      <c r="D29" s="107"/>
-      <c r="E29" s="107"/>
-      <c r="F29" s="107"/>
-      <c r="G29" s="107"/>
-      <c r="H29" s="107"/>
-      <c r="I29" s="103"/>
+      <c r="B29" s="126"/>
+      <c r="C29" s="103"/>
+      <c r="D29" s="103"/>
+      <c r="E29" s="103"/>
+      <c r="F29" s="103"/>
+      <c r="G29" s="103"/>
+      <c r="H29" s="103"/>
+      <c r="I29" s="121"/>
     </row>
     <row r="30" spans="1:11" s="20" customFormat="1" ht="25" customHeight="1">
       <c r="A30" s="21"/>
-      <c r="B30" s="108"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="107"/>
-      <c r="F30" s="107"/>
-      <c r="G30" s="107"/>
-      <c r="H30" s="107"/>
-      <c r="I30" s="103"/>
+      <c r="B30" s="110"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="103"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="103"/>
+      <c r="G30" s="103"/>
+      <c r="H30" s="103"/>
+      <c r="I30" s="121"/>
     </row>
     <row r="31" spans="1:11" s="20" customFormat="1" ht="25" customHeight="1">
       <c r="A31" s="21"/>
-      <c r="B31" s="109"/>
-      <c r="C31" s="110"/>
-      <c r="D31" s="110"/>
-      <c r="E31" s="110"/>
-      <c r="F31" s="110"/>
-      <c r="G31" s="110"/>
-      <c r="H31" s="110"/>
-      <c r="I31" s="105"/>
+      <c r="B31" s="113"/>
+      <c r="C31" s="122"/>
+      <c r="D31" s="122"/>
+      <c r="E31" s="122"/>
+      <c r="F31" s="122"/>
+      <c r="G31" s="122"/>
+      <c r="H31" s="122"/>
+      <c r="I31" s="114"/>
     </row>
     <row r="32" spans="1:11" s="20" customFormat="1" ht="20" customHeight="1">
       <c r="A32" s="21"/>
@@ -1870,13 +1825,13 @@
     </row>
     <row r="33" spans="1:9" ht="35" customHeight="1">
       <c r="B33" s="50" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C33" s="45"/>
       <c r="D33" s="51"/>
       <c r="E33" s="52"/>
       <c r="F33" s="50" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G33" s="45"/>
       <c r="H33" s="51"/>
@@ -1916,17 +1871,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:E21"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="B14:E15"/>
-    <mergeCell ref="F24:G24"/>
     <mergeCell ref="F26:G26"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="B29:I31"/>
@@ -1940,6 +1884,17 @@
     <mergeCell ref="H26:I26"/>
     <mergeCell ref="F25:G25"/>
     <mergeCell ref="H25:I25"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:E21"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B14:E15"/>
+    <mergeCell ref="F24:G24"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="3">
@@ -1949,6 +1904,5 @@
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="67" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>